<commit_message>
Add PDF download, text extraction, source_page field, search on text
- scrape_cy4gate.py: download all PDFs into 2024/2025/2026 folders,
  extract full text with PyMuPDF, add source_page URL per record
- comunicati.json / data.js: updated with testo and source_page fields
- index.html: remove CY4GATE from topbar, search now includes pdf text

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cy4gate_comunicati_stampa.xlsx
+++ b/cy4gate_comunicati_stampa.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comunicati Stampa" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Comunicati Stampa'!$A$1:$E$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Comunicati Stampa'!$A$1:$F$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:F84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -461,6 +461,7 @@
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="80" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -489,6 +490,11 @@
           <t>Link</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Source Page</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -512,6 +518,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-3/</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -535,6 +546,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-3/</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -558,6 +574,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-3/</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -581,6 +602,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-3/</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -604,6 +630,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-3/</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -627,6 +658,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-3/</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -650,6 +686,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-3/</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -673,6 +714,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -696,6 +742,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -719,6 +770,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -742,6 +798,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -765,6 +826,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -788,6 +854,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -811,6 +882,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -834,6 +910,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -857,6 +938,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -880,6 +966,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -903,6 +994,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -926,6 +1022,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -949,6 +1050,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -972,6 +1078,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -995,6 +1106,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1018,6 +1134,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1041,6 +1162,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1064,6 +1190,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1087,6 +1218,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1110,6 +1246,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1133,6 +1274,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1156,6 +1302,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1179,6 +1330,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -1202,6 +1358,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1225,6 +1386,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -1248,6 +1414,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1271,6 +1442,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -1294,6 +1470,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1317,6 +1498,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2025/</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -1340,6 +1526,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1363,6 +1554,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -1386,6 +1582,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1409,6 +1610,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -1432,6 +1638,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1455,6 +1666,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -1478,6 +1694,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1501,6 +1722,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -1524,6 +1750,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1547,6 +1778,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -1570,6 +1806,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1593,6 +1834,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -1616,6 +1862,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1639,6 +1890,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -1662,6 +1918,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1685,6 +1946,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F53" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -1708,6 +1974,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1731,6 +2002,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -1754,6 +2030,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1777,6 +2058,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F57" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -1800,6 +2086,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1823,6 +2114,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F59" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -1846,6 +2142,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1869,6 +2170,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F61" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -1892,6 +2198,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1915,6 +2226,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F63" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -1938,6 +2254,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1961,6 +2282,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F65" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -1984,6 +2310,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2007,6 +2338,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F67" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -2030,6 +2366,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -2049,6 +2390,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F69" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -2072,6 +2418,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2095,6 +2446,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F71" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -2118,6 +2474,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -2141,6 +2502,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F73" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -2164,6 +2530,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -2187,6 +2558,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F75" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -2210,6 +2586,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -2233,6 +2614,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F77" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -2256,6 +2642,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -2279,6 +2670,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F79" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -2302,6 +2698,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -2325,6 +2726,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F81" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -2348,6 +2754,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -2371,6 +2782,11 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F83" s="8" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -2394,93 +2810,181 @@
           <t>Apri PDF</t>
         </is>
       </c>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>https://www.cy4gate.com/company/investor-relations/financial-press-releases/year-2024/</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E84"/>
+  <autoFilter ref="A1:F84"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F48" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F57" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F58" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F59" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F80" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F81" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E83" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F83" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E84" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F84" r:id="rId166"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>